<commit_message>
e2e testing and frontend fix
</commit_message>
<xml_diff>
--- a/TestingPlan.xlsx
+++ b/TestingPlan.xlsx
@@ -184,49 +184,49 @@
     <author>TennisComp</author>
   </authors>
   <commentList>
-    <comment ref="J79" authorId="0" shapeId="0">
-      <text>
-        <t>Checked in Chrome on 28 Sep 2026 against the seeded test data.</t>
-      </text>
-    </comment>
-    <comment ref="J81" authorId="0" shapeId="0">
-      <text>
-        <t>Checked in Chrome on 28 Sep 2026 against the seeded test data.</t>
-      </text>
-    </comment>
     <comment ref="J83" authorId="0" shapeId="0">
       <text>
-        <t>Checked in Chrome on 28 Sep 2026 against the seeded test data.</t>
+        <t>Automated with Playwright; the testing steps are what the script does, so they can also be followed by hand.</t>
       </text>
     </comment>
     <comment ref="J85" authorId="0" shapeId="0">
       <text>
-        <t>Checked in Chrome on 28 Sep 2026 against the seeded test data.</t>
+        <t>Automated with Playwright; the testing steps are what the script does, so they can also be followed by hand.</t>
       </text>
     </comment>
     <comment ref="J87" authorId="0" shapeId="0">
       <text>
-        <t>Checked in Chrome on 28 Sep 2026 against the seeded test data.</t>
+        <t>Automated with Playwright; the testing steps are what the script does, so they can also be followed by hand.</t>
       </text>
     </comment>
     <comment ref="J89" authorId="0" shapeId="0">
       <text>
-        <t>Checked in Chrome on 28 Sep 2026 against the seeded test data.</t>
+        <t>Automated with Playwright; the testing steps are what the script does, so they can also be followed by hand.</t>
       </text>
     </comment>
     <comment ref="J91" authorId="0" shapeId="0">
       <text>
-        <t>Checked in Chrome on 28 Sep 2026 against the seeded test data.</t>
+        <t>Automated with Playwright; the testing steps are what the script does, so they can also be followed by hand.</t>
       </text>
     </comment>
     <comment ref="J93" authorId="0" shapeId="0">
       <text>
-        <t>Checked in Chrome on 28 Sep 2026 against the seeded test data.</t>
+        <t>Automated with Playwright; the testing steps are what the script does, so they can also be followed by hand.</t>
       </text>
     </comment>
     <comment ref="J95" authorId="0" shapeId="0">
       <text>
-        <t>Checked in Chrome on 28 Sep 2026 against the seeded test data.</t>
+        <t>Automated with Playwright; the testing steps are what the script does, so they can also be followed by hand.</t>
+      </text>
+    </comment>
+    <comment ref="J97" authorId="0" shapeId="0">
+      <text>
+        <t>Automated with Playwright; the testing steps are what the script does, so they can also be followed by hand.</t>
+      </text>
+    </comment>
+    <comment ref="J99" authorId="0" shapeId="0">
+      <text>
+        <t>Automated with Playwright; the testing steps are what the script does, so they can also be followed by hand.</t>
       </text>
     </comment>
   </commentList>
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -545,7 +545,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Backend tests use Node's built-in test runner with @nestjs/testing; frontend tests use Vitest, with React Testing Library for rendering components. Unit = one function or service with a fake database; Integration = a real HTTP route or a rendered component; End to end = the whole app in a browser, done manually.</t>
+          <t>Backend tests use Node's built-in test runner with @nestjs/testing; frontend tests use Vitest, with React Testing Library for rendering components. End to end tests use Playwright. Unit = one function or service with a fake database; Integration = a real HTTP route or a rendered component; End to end = the whole app in a real browser against a real, seeded database.</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>npm test  (project root: runs backend then frontend; no database needed)</t>
+          <t>npm test  (unit + integration, no database needed)   ·   npm run test:e2e  (end to end; database running and seeded)</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>28 Sep 2026: backend 44/44 passed, frontend 20/20 passed. Also runs automatically on every push and pull request (GitHub Actions).</t>
+          <t>28 Sep 2026: backend 44/44, frontend 23/23, end to end 9/9 passed. All of them run automatically on every push and pull request (GitHub Actions).</t>
         </is>
       </c>
     </row>
@@ -2195,97 +2195,97 @@
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="3" t="n"/>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>FE-007</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>npm test</t>
+        </is>
+      </c>
+      <c r="D51" s="4">
+        <f>PROPER(G51)</f>
+        <v/>
+      </c>
+      <c r="E51" s="4">
+        <f>PROPER(H51)</f>
+        <v/>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>frontend/tests/formatters.test.ts</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>a utr percentile is shown as a top percentage, never top 0 percent</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="n"/>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>Test type</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Execution Type</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Objective</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>Setup</t>
         </is>
       </c>
-      <c r="G52" s="2" t="n"/>
-      <c r="H52" s="2" t="n"/>
-      <c r="I52" s="2" t="n"/>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="G53" s="2" t="n"/>
+      <c r="H53" s="2" t="n"/>
+      <c r="I53" s="2" t="n"/>
+      <c r="J53" s="2" t="inlineStr">
         <is>
           <t>Done?</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="7" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
         <is>
           <t>Integration</t>
         </is>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B54" s="8" t="inlineStr">
         <is>
           <t>I-AUTH-001</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>npm test</t>
-        </is>
-      </c>
-      <c r="D53" s="8">
-        <f>PROPER(G53)</f>
-        <v/>
-      </c>
-      <c r="E53" s="8">
-        <f>PROPER(H53)</f>
-        <v/>
-      </c>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>POST /auth/login (backend/test/auth.test.cjs)</t>
-        </is>
-      </c>
-      <c r="G53" s="8" t="inlineStr">
-        <is>
-          <t>login answers 200 for both success and failure</t>
-        </is>
-      </c>
-      <c r="H53" s="8" t="inlineStr">
-        <is>
-          <t>account is already created</t>
-        </is>
-      </c>
-      <c r="I53" s="9" t="n"/>
-      <c r="J53" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="n"/>
-      <c r="B54" s="8" t="inlineStr">
-        <is>
-          <t>I-AUTH-002</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
@@ -2308,12 +2308,12 @@
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>login with an empty body fails without crashing</t>
+          <t>login answers 200 for both success and failure</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>account is already created</t>
         </is>
       </c>
       <c r="I54" s="9" t="n"/>
@@ -2324,64 +2324,64 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="n"/>
-      <c r="B55" s="6" t="n"/>
-      <c r="C55" s="6" t="n"/>
-      <c r="D55" s="6" t="n"/>
-      <c r="E55" s="6" t="n"/>
-      <c r="F55" s="6" t="n"/>
-      <c r="G55" s="6" t="n"/>
-      <c r="H55" s="6" t="n"/>
-      <c r="I55" s="6" t="n"/>
-      <c r="J55" s="6" t="n"/>
+      <c r="A55" s="7" t="n"/>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>I-AUTH-002</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>npm test</t>
+        </is>
+      </c>
+      <c r="D55" s="8">
+        <f>PROPER(G55)</f>
+        <v/>
+      </c>
+      <c r="E55" s="8">
+        <f>PROPER(H55)</f>
+        <v/>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>POST /auth/login (backend/test/auth.test.cjs)</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>login with an empty body fails without crashing</t>
+        </is>
+      </c>
+      <c r="H55" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I55" s="9" t="n"/>
+      <c r="J55" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="n"/>
-      <c r="B56" s="8" t="inlineStr">
-        <is>
-          <t>I-DASH-001</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>npm test</t>
-        </is>
-      </c>
-      <c r="D56" s="8">
-        <f>PROPER(G56)</f>
-        <v/>
-      </c>
-      <c r="E56" s="8">
-        <f>PROPER(H56)</f>
-        <v/>
-      </c>
-      <c r="F56" s="8" t="inlineStr">
-        <is>
-          <t>GET /api/v1/player-dashboard (backend/test/dashboard.test.cjs)</t>
-        </is>
-      </c>
-      <c r="G56" s="8" t="inlineStr">
-        <is>
-          <t>dashboard loads for a normalised email and reads only needed fields</t>
-        </is>
-      </c>
-      <c r="H56" s="8" t="inlineStr">
-        <is>
-          <t>account is linked to a player</t>
-        </is>
-      </c>
-      <c r="I56" s="9" t="n"/>
-      <c r="J56" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="A56" s="6" t="n"/>
+      <c r="B56" s="6" t="n"/>
+      <c r="C56" s="6" t="n"/>
+      <c r="D56" s="6" t="n"/>
+      <c r="E56" s="6" t="n"/>
+      <c r="F56" s="6" t="n"/>
+      <c r="G56" s="6" t="n"/>
+      <c r="H56" s="6" t="n"/>
+      <c r="I56" s="6" t="n"/>
+      <c r="J56" s="6" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n"/>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>I-DASH-002</t>
+          <t>I-DASH-001</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
@@ -2399,17 +2399,17 @@
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>GET /api/v1/player-dashboard</t>
+          <t>GET /api/v1/player-dashboard (backend/test/dashboard.test.cjs)</t>
         </is>
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>another email loads a different profile, teams and fixtures</t>
+          <t>dashboard loads for a normalised email and reads only needed fields</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>two players exist</t>
+          <t>account is linked to a player</t>
         </is>
       </c>
       <c r="I57" s="9" t="n"/>
@@ -2423,7 +2423,7 @@
       <c r="A58" s="7" t="n"/>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>I-DASH-003</t>
+          <t>I-DASH-002</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
@@ -2446,12 +2446,12 @@
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>missing account and missing profile give different not found errors</t>
+          <t>another email loads a different profile, teams and fixtures</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>two players exist</t>
         </is>
       </c>
       <c r="I58" s="9" t="n"/>
@@ -2465,7 +2465,7 @@
       <c r="A59" s="7" t="n"/>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>I-DASH-004</t>
+          <t>I-DASH-003</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
@@ -2483,17 +2483,17 @@
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>GET /api/v1/player-dashboard/results</t>
+          <t>GET /api/v1/player-dashboard</t>
         </is>
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>result scores and outcomes are from the player side</t>
+          <t>missing account and missing profile give different not found errors</t>
         </is>
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>rubber is finalised</t>
+          <t>none</t>
         </is>
       </c>
       <c r="I59" s="9" t="n"/>
@@ -2507,7 +2507,7 @@
       <c r="A60" s="7" t="n"/>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>I-DASH-005</t>
+          <t>I-DASH-004</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
@@ -2525,17 +2525,17 @@
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>GET /api/v1/player-dashboard/schedule</t>
+          <t>GET /api/v1/player-dashboard/results</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>page cursors continue without repeats and cannot switch account</t>
+          <t>result scores and outcomes are from the player side</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t>player has more than one page of fixtures</t>
+          <t>rubber is finalised</t>
         </is>
       </c>
       <c r="I60" s="9" t="n"/>
@@ -2549,7 +2549,7 @@
       <c r="A61" s="7" t="n"/>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>I-DASH-006</t>
+          <t>I-DASH-005</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
@@ -2572,12 +2572,12 @@
       </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
-          <t>full schedule includes old and cancelled fixtures; date ranges work</t>
+          <t>page cursors continue without repeats and cannot switch account</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>fixtures in several states</t>
+          <t>player has more than one page of fixtures</t>
         </is>
       </c>
       <c r="I61" s="9" t="n"/>
@@ -2591,7 +2591,7 @@
       <c r="A62" s="7" t="n"/>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>I-DASH-007</t>
+          <t>I-DASH-006</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
@@ -2609,17 +2609,17 @@
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>GET /api/v1/player-dashboard/notifications</t>
+          <t>GET /api/v1/player-dashboard/schedule</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>notifications belong to the player, newest first, with an unread count</t>
+          <t>full schedule includes old and cancelled fixtures; date ranges work</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>player has notifications</t>
+          <t>fixtures in several states</t>
         </is>
       </c>
       <c r="I62" s="9" t="n"/>
@@ -2633,7 +2633,7 @@
       <c r="A63" s="7" t="n"/>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>I-DASH-008</t>
+          <t>I-DASH-007</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
@@ -2651,17 +2651,17 @@
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>GET /api/v1/player-dashboard</t>
+          <t>GET /api/v1/player-dashboard/notifications</t>
         </is>
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>bad queries and outages never return empty data or private errors</t>
+          <t>notifications belong to the player, newest first, with an unread count</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>player has notifications</t>
         </is>
       </c>
       <c r="I63" s="9" t="n"/>
@@ -2675,7 +2675,7 @@
       <c r="A64" s="7" t="n"/>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>I-DASH-009</t>
+          <t>I-DASH-008</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
@@ -2698,12 +2698,12 @@
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>email lookup is refused in production</t>
+          <t>bad queries and outages never return empty data or private errors</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>node env is production</t>
+          <t>none</t>
         </is>
       </c>
       <c r="I64" s="9" t="n"/>
@@ -2714,64 +2714,64 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="n"/>
-      <c r="B65" s="6" t="n"/>
-      <c r="C65" s="6" t="n"/>
-      <c r="D65" s="6" t="n"/>
-      <c r="E65" s="6" t="n"/>
-      <c r="F65" s="6" t="n"/>
-      <c r="G65" s="6" t="n"/>
-      <c r="H65" s="6" t="n"/>
-      <c r="I65" s="6" t="n"/>
-      <c r="J65" s="6" t="n"/>
+      <c r="A65" s="7" t="n"/>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>I-DASH-009</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>npm test</t>
+        </is>
+      </c>
+      <c r="D65" s="8">
+        <f>PROPER(G65)</f>
+        <v/>
+      </c>
+      <c r="E65" s="8">
+        <f>PROPER(H65)</f>
+        <v/>
+      </c>
+      <c r="F65" s="8" t="inlineStr">
+        <is>
+          <t>GET /api/v1/player-dashboard</t>
+        </is>
+      </c>
+      <c r="G65" s="8" t="inlineStr">
+        <is>
+          <t>email lookup is refused in production</t>
+        </is>
+      </c>
+      <c r="H65" s="8" t="inlineStr">
+        <is>
+          <t>node env is production</t>
+        </is>
+      </c>
+      <c r="I65" s="9" t="n"/>
+      <c r="J65" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="7" t="n"/>
-      <c r="B66" s="8" t="inlineStr">
-        <is>
-          <t>I-PLAYER-001</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>npm test</t>
-        </is>
-      </c>
-      <c r="D66" s="8">
-        <f>PROPER(G66)</f>
-        <v/>
-      </c>
-      <c r="E66" s="8">
-        <f>PROPER(H66)</f>
-        <v/>
-      </c>
-      <c r="F66" s="8" t="inlineStr">
-        <is>
-          <t>GET /api/v1/player/* (backend/test/player.test.cjs)</t>
-        </is>
-      </c>
-      <c r="G66" s="8" t="inlineStr">
-        <is>
-          <t>every player route returns data for a valid email</t>
-        </is>
-      </c>
-      <c r="H66" s="8" t="inlineStr">
-        <is>
-          <t>account is linked to a player</t>
-        </is>
-      </c>
-      <c r="I66" s="9" t="n"/>
-      <c r="J66" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="A66" s="6" t="n"/>
+      <c r="B66" s="6" t="n"/>
+      <c r="C66" s="6" t="n"/>
+      <c r="D66" s="6" t="n"/>
+      <c r="E66" s="6" t="n"/>
+      <c r="F66" s="6" t="n"/>
+      <c r="G66" s="6" t="n"/>
+      <c r="H66" s="6" t="n"/>
+      <c r="I66" s="6" t="n"/>
+      <c r="J66" s="6" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="n"/>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>I-PLAYER-002</t>
+          <t>I-PLAYER-001</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
@@ -2789,12 +2789,12 @@
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>GET /api/v1/player/fixtures</t>
+          <t>GET /api/v1/player/* (backend/test/player.test.cjs)</t>
         </is>
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>the email is normalised before lookup</t>
+          <t>every player route returns data for a valid email</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr">
@@ -2813,7 +2813,7 @@
       <c r="A68" s="7" t="n"/>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>I-PLAYER-003</t>
+          <t>I-PLAYER-002</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
@@ -2831,17 +2831,17 @@
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>GET /api/v1/player/*</t>
+          <t>GET /api/v1/player/fixtures</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>a missing or malformed email, or a bad team id, returns 400</t>
+          <t>the email is normalised before lookup</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>account is linked to a player</t>
         </is>
       </c>
       <c r="I68" s="9" t="n"/>
@@ -2855,7 +2855,7 @@
       <c r="A69" s="7" t="n"/>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>I-PLAYER-004</t>
+          <t>I-PLAYER-003</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
@@ -2878,12 +2878,12 @@
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>player routes are refused in production</t>
+          <t>a missing or malformed email, or a bad team id, returns 400</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr">
         <is>
-          <t>node env is production</t>
+          <t>none</t>
         </is>
       </c>
       <c r="I69" s="9" t="n"/>
@@ -2894,64 +2894,64 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="6" t="n"/>
-      <c r="B70" s="6" t="n"/>
-      <c r="C70" s="6" t="n"/>
-      <c r="D70" s="6" t="n"/>
-      <c r="E70" s="6" t="n"/>
-      <c r="F70" s="6" t="n"/>
-      <c r="G70" s="6" t="n"/>
-      <c r="H70" s="6" t="n"/>
-      <c r="I70" s="6" t="n"/>
-      <c r="J70" s="6" t="n"/>
+      <c r="A70" s="7" t="n"/>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>I-PLAYER-004</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>npm test</t>
+        </is>
+      </c>
+      <c r="D70" s="8">
+        <f>PROPER(G70)</f>
+        <v/>
+      </c>
+      <c r="E70" s="8">
+        <f>PROPER(H70)</f>
+        <v/>
+      </c>
+      <c r="F70" s="8" t="inlineStr">
+        <is>
+          <t>GET /api/v1/player/*</t>
+        </is>
+      </c>
+      <c r="G70" s="8" t="inlineStr">
+        <is>
+          <t>player routes are refused in production</t>
+        </is>
+      </c>
+      <c r="H70" s="8" t="inlineStr">
+        <is>
+          <t>node env is production</t>
+        </is>
+      </c>
+      <c r="I70" s="9" t="n"/>
+      <c r="J70" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="n"/>
-      <c r="B71" s="8" t="inlineStr">
-        <is>
-          <t>I-FE-001</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>npm test</t>
-        </is>
-      </c>
-      <c r="D71" s="8">
-        <f>PROPER(G71)</f>
-        <v/>
-      </c>
-      <c r="E71" s="8">
-        <f>PROPER(H71)</f>
-        <v/>
-      </c>
-      <c r="F71" s="8" t="inlineStr">
-        <is>
-          <t>api adapters (frontend/tests/api-adapters.test.ts)</t>
-        </is>
-      </c>
-      <c r="G71" s="8" t="inlineStr">
-        <is>
-          <t>logged out visitors get the sample without calling the backend</t>
-        </is>
-      </c>
-      <c r="H71" s="8" t="inlineStr">
-        <is>
-          <t>nobody is logged in</t>
-        </is>
-      </c>
-      <c r="I71" s="9" t="n"/>
-      <c r="J71" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="A71" s="6" t="n"/>
+      <c r="B71" s="6" t="n"/>
+      <c r="C71" s="6" t="n"/>
+      <c r="D71" s="6" t="n"/>
+      <c r="E71" s="6" t="n"/>
+      <c r="F71" s="6" t="n"/>
+      <c r="G71" s="6" t="n"/>
+      <c r="H71" s="6" t="n"/>
+      <c r="I71" s="6" t="n"/>
+      <c r="J71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n"/>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>I-FE-002</t>
+          <t>I-FE-001</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
@@ -2974,12 +2974,12 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>logged in players always get backend data, never the sample</t>
+          <t>logged out visitors get the sample without calling the backend</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
         <is>
-          <t>player is logged in</t>
+          <t>nobody is logged in</t>
         </is>
       </c>
       <c r="I72" s="9" t="n"/>
@@ -2993,7 +2993,7 @@
       <c r="A73" s="7" t="n"/>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>I-FE-003</t>
+          <t>I-FE-002</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>another team or a bad team id shows not found</t>
+          <t>logged in players always get backend data, never the sample</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -3032,64 +3032,64 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="6" t="n"/>
-      <c r="B74" s="6" t="n"/>
-      <c r="C74" s="6" t="n"/>
-      <c r="D74" s="6" t="n"/>
-      <c r="E74" s="6" t="n"/>
-      <c r="F74" s="6" t="n"/>
-      <c r="G74" s="6" t="n"/>
-      <c r="H74" s="6" t="n"/>
-      <c r="I74" s="6" t="n"/>
-      <c r="J74" s="6" t="n"/>
+      <c r="A74" s="7" t="n"/>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>I-FE-003</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>npm test</t>
+        </is>
+      </c>
+      <c r="D74" s="8">
+        <f>PROPER(G74)</f>
+        <v/>
+      </c>
+      <c r="E74" s="8">
+        <f>PROPER(H74)</f>
+        <v/>
+      </c>
+      <c r="F74" s="8" t="inlineStr">
+        <is>
+          <t>api adapters (frontend/tests/api-adapters.test.ts)</t>
+        </is>
+      </c>
+      <c r="G74" s="8" t="inlineStr">
+        <is>
+          <t>another team or a bad team id shows not found</t>
+        </is>
+      </c>
+      <c r="H74" s="8" t="inlineStr">
+        <is>
+          <t>player is logged in</t>
+        </is>
+      </c>
+      <c r="I74" s="9" t="n"/>
+      <c r="J74" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="7" t="n"/>
-      <c r="B75" s="8" t="inlineStr">
-        <is>
-          <t>I-UI-001</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>npm test</t>
-        </is>
-      </c>
-      <c r="D75" s="8">
-        <f>PROPER(G75)</f>
-        <v/>
-      </c>
-      <c r="E75" s="8">
-        <f>PROPER(H75)</f>
-        <v/>
-      </c>
-      <c r="F75" s="8" t="inlineStr">
-        <is>
-          <t>render LoginPage (frontend/tests/login-page.test.tsx)</t>
-        </is>
-      </c>
-      <c r="G75" s="8" t="inlineStr">
-        <is>
-          <t>the login form shows an error for a wrong password or an unreachable server, and opens the dashboard on success</t>
-        </is>
-      </c>
-      <c r="H75" s="8" t="inlineStr">
-        <is>
-          <t>backend answers are simulated</t>
-        </is>
-      </c>
-      <c r="I75" s="9" t="n"/>
-      <c r="J75" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="A75" s="6" t="n"/>
+      <c r="B75" s="6" t="n"/>
+      <c r="C75" s="6" t="n"/>
+      <c r="D75" s="6" t="n"/>
+      <c r="E75" s="6" t="n"/>
+      <c r="F75" s="6" t="n"/>
+      <c r="G75" s="6" t="n"/>
+      <c r="H75" s="6" t="n"/>
+      <c r="I75" s="6" t="n"/>
+      <c r="J75" s="6" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="n"/>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>I-UI-002</t>
+          <t>I-UI-001</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
@@ -3107,12 +3107,12 @@
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>render NotificationPanel (frontend/tests/notification-panel.test.tsx)</t>
+          <t>render LoginPage (frontend/tests/login-page.test.tsx)</t>
         </is>
       </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>the notifications card lists items with the date line, links fixtures, and view all loads the full list</t>
+          <t>the login form shows an error for a wrong password or an unreachable server, and opens the dashboard on success</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
@@ -3127,198 +3127,236 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="7" t="n"/>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>I-UI-002</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>npm test</t>
+        </is>
+      </c>
+      <c r="D77" s="8">
+        <f>PROPER(G77)</f>
+        <v/>
+      </c>
+      <c r="E77" s="8">
+        <f>PROPER(H77)</f>
+        <v/>
+      </c>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>render NotificationPanel (frontend/tests/notification-panel.test.tsx)</t>
+        </is>
+      </c>
+      <c r="G77" s="8" t="inlineStr">
+        <is>
+          <t>the notifications card lists items with the date line, links fixtures, and view all loads the full list</t>
+        </is>
+      </c>
+      <c r="H77" s="8" t="inlineStr">
+        <is>
+          <t>backend answers are simulated</t>
+        </is>
+      </c>
+      <c r="I77" s="9" t="n"/>
+      <c r="J77" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
+      <c r="A78" s="7" t="n"/>
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>I-UI-003</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>npm test</t>
+        </is>
+      </c>
+      <c r="D78" s="8">
+        <f>PROPER(G78)</f>
+        <v/>
+      </c>
+      <c r="E78" s="8">
+        <f>PROPER(H78)</f>
+        <v/>
+      </c>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>render CareerSummary (frontend/tests/career-summary.test.tsx)</t>
+        </is>
+      </c>
+      <c r="G78" s="8" t="inlineStr">
+        <is>
+          <t>the career summary shows win percentage, titles, and the best rank with its ranking group</t>
+        </is>
+      </c>
+      <c r="H78" s="8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I78" s="9" t="n"/>
+      <c r="J78" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n"/>
+      <c r="B79" s="6" t="n"/>
+      <c r="C79" s="6" t="n"/>
+      <c r="D79" s="6" t="n"/>
+      <c r="E79" s="6" t="n"/>
+      <c r="F79" s="6" t="n"/>
+      <c r="G79" s="6" t="n"/>
+      <c r="H79" s="6" t="n"/>
+      <c r="I79" s="6" t="n"/>
+      <c r="J79" s="6" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="7" t="n"/>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>I-DB-001</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>npm test</t>
+        </is>
+      </c>
+      <c r="D80" s="8">
+        <f>PROPER(G80)</f>
+        <v/>
+      </c>
+      <c r="E80" s="8">
+        <f>PROPER(H80)</f>
+        <v/>
+      </c>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>CI end-to-end job (.github/workflows/ci.yml)</t>
+        </is>
+      </c>
+      <c r="G80" s="8" t="inlineStr">
+        <is>
+          <t>a brand new empty database migrates and seeds without errors</t>
+        </is>
+      </c>
+      <c r="H80" s="8" t="inlineStr">
+        <is>
+          <t>empty postgres database</t>
+        </is>
+      </c>
+      <c r="I80" s="9" t="n"/>
+      <c r="J80" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>Test type</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>Test ID (User story code)</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Execution Type</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="D82" s="2" t="inlineStr">
         <is>
           <t>Objective</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr">
+      <c r="E82" s="2" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
+      <c r="F82" s="2" t="inlineStr">
         <is>
           <t>Setup</t>
         </is>
       </c>
-      <c r="G78" s="2" t="n"/>
-      <c r="H78" s="2" t="n"/>
-      <c r="I78" s="2" t="inlineStr">
+      <c r="G82" s="2" t="n"/>
+      <c r="H82" s="2" t="n"/>
+      <c r="I82" s="2" t="inlineStr">
         <is>
           <t>Testing steps</t>
         </is>
       </c>
-      <c r="J78" s="2" t="inlineStr">
+      <c r="J82" s="2" t="inlineStr">
         <is>
           <t>Done?</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="10" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="10" t="inlineStr">
         <is>
           <t>End to end</t>
         </is>
       </c>
-      <c r="B79" s="11" t="inlineStr">
+      <c r="B83" s="11" t="inlineStr">
         <is>
           <t>E2E-001</t>
         </is>
       </c>
-      <c r="C79" s="11" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D79" s="11">
-        <f>PROPER(G79)</f>
-        <v/>
-      </c>
-      <c r="E79" s="11">
-        <f>PROPER(H79)</f>
-        <v/>
-      </c>
-      <c r="F79" s="12" t="inlineStr">
-        <is>
-          <t>• Database running and seeded (npm run seed:competition)
-• npm run dev:backend and npm run dev:frontend
-• Open http://localhost:5173</t>
-        </is>
-      </c>
-      <c r="G79" s="11" t="inlineStr">
+      <c r="C83" s="11" t="inlineStr">
+        <is>
+          <t>npm run test:e2e</t>
+        </is>
+      </c>
+      <c r="D83" s="11">
+        <f>PROPER(G83)</f>
+        <v/>
+      </c>
+      <c r="E83" s="11">
+        <f>PROPER(H83)</f>
+        <v/>
+      </c>
+      <c r="F83" s="12" t="inlineStr">
+        <is>
+          <t>e2e/player-journeys.spec.ts
+• Database running and seeded (npm run seed:competition)
+• npm run test:e2e starts the backend and frontend if they are not running</t>
+        </is>
+      </c>
+      <c r="G83" s="11" t="inlineStr">
         <is>
           <t>log in and see my profile</t>
         </is>
       </c>
-      <c r="H79" s="11" t="inlineStr">
+      <c r="H83" s="11" t="inlineStr">
         <is>
           <t>test data is seeded</t>
         </is>
       </c>
-      <c r="I79" s="12" t="inlineStr">
+      <c r="I83" s="12" t="inlineStr">
         <is>
           <t>• Log in as chloe.cooper005@players.example / WaverleyDev#2026
 • Check name, age, clubs, association and teams on the profile card
 • Check Current UTR is 5.35 and Win % is 59.3%</t>
         </is>
       </c>
-      <c r="J79" s="11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="13" t="n"/>
-      <c r="B81" s="11" t="inlineStr">
-        <is>
-          <t>E2E-002</t>
-        </is>
-      </c>
-      <c r="C81" s="11" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D81" s="11">
-        <f>PROPER(G81)</f>
-        <v/>
-      </c>
-      <c r="E81" s="11">
-        <f>PROPER(H81)</f>
-        <v/>
-      </c>
-      <c r="F81" s="12" t="inlineStr">
-        <is>
-          <t>• Database running and seeded (npm run seed:competition)
-• npm run dev:backend and npm run dev:frontend
-• Open http://localhost:5173</t>
-        </is>
-      </c>
-      <c r="G81" s="11" t="inlineStr">
-        <is>
-          <t>log in with a wrong password</t>
-        </is>
-      </c>
-      <c r="H81" s="11" t="inlineStr">
-        <is>
-          <t>test data is seeded</t>
-        </is>
-      </c>
-      <c r="I81" s="12" t="inlineStr">
-        <is>
-          <t>• Enter chloe.cooper005@players.example with a wrong password
-• Check the message Incorrect email or password appears and you stay on the login page</t>
-        </is>
-      </c>
-      <c r="J81" s="11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="13" t="n"/>
-      <c r="B83" s="11" t="inlineStr">
-        <is>
-          <t>E2E-003</t>
-        </is>
-      </c>
-      <c r="C83" s="11" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D83" s="11">
-        <f>PROPER(G83)</f>
-        <v/>
-      </c>
-      <c r="E83" s="11">
-        <f>PROPER(H83)</f>
-        <v/>
-      </c>
-      <c r="F83" s="12" t="inlineStr">
-        <is>
-          <t>• Database running and seeded (npm run seed:competition)
-• npm run dev:backend and npm run dev:frontend
-• Open http://localhost:5173</t>
-        </is>
-      </c>
-      <c r="G83" s="11" t="inlineStr">
-        <is>
-          <t>see my notifications</t>
-        </is>
-      </c>
-      <c r="H83" s="11" t="inlineStr">
-        <is>
-          <t>test data is seeded</t>
-        </is>
-      </c>
-      <c r="I83" s="12" t="inlineStr">
-        <is>
-          <t>• Log in as chloe.cooper005@players.example / WaverleyDev#2026
-• Check the Notifications card lists 3 notifications with icons and times
-• Check the date change shows Sep 26 → Sep 27, 2026
-• Click a notification and check the fixture details open</t>
-        </is>
-      </c>
       <c r="J83" s="11" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3329,12 +3367,12 @@
       <c r="A85" s="13" t="n"/>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>E2E-004</t>
+          <t>E2E-002</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>npm run test:e2e</t>
         </is>
       </c>
       <c r="D85" s="11">
@@ -3347,22 +3385,122 @@
       </c>
       <c r="F85" s="12" t="inlineStr">
         <is>
-          <t>• Database running and seeded (npm run seed:competition)
-• npm run dev:backend and npm run dev:frontend
-• Open http://localhost:5173</t>
+          <t>e2e/player-journeys.spec.ts
+• Database running and seeded (npm run seed:competition)
+• npm run test:e2e starts the backend and frontend if they are not running</t>
         </is>
       </c>
       <c r="G85" s="11" t="inlineStr">
         <is>
+          <t>log in with a wrong password</t>
+        </is>
+      </c>
+      <c r="H85" s="11" t="inlineStr">
+        <is>
+          <t>test data is seeded</t>
+        </is>
+      </c>
+      <c r="I85" s="12" t="inlineStr">
+        <is>
+          <t>• Enter chloe.cooper005@players.example with a wrong password
+• Check the message Incorrect email or password appears and you stay on the login page</t>
+        </is>
+      </c>
+      <c r="J85" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="13" t="n"/>
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>E2E-003</t>
+        </is>
+      </c>
+      <c r="C87" s="11" t="inlineStr">
+        <is>
+          <t>npm run test:e2e</t>
+        </is>
+      </c>
+      <c r="D87" s="11">
+        <f>PROPER(G87)</f>
+        <v/>
+      </c>
+      <c r="E87" s="11">
+        <f>PROPER(H87)</f>
+        <v/>
+      </c>
+      <c r="F87" s="12" t="inlineStr">
+        <is>
+          <t>e2e/player-journeys.spec.ts
+• Database running and seeded (npm run seed:competition)
+• npm run test:e2e starts the backend and frontend if they are not running</t>
+        </is>
+      </c>
+      <c r="G87" s="11" t="inlineStr">
+        <is>
+          <t>see my notifications</t>
+        </is>
+      </c>
+      <c r="H87" s="11" t="inlineStr">
+        <is>
+          <t>test data is seeded</t>
+        </is>
+      </c>
+      <c r="I87" s="12" t="inlineStr">
+        <is>
+          <t>• Log in as chloe.cooper005@players.example / WaverleyDev#2026
+• Check the Notifications card lists 3 notifications
+• Check the date change shows Sep 26 → Sep 27, 2026
+• Click a notification and check the fixture details open</t>
+        </is>
+      </c>
+      <c r="J87" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="13" t="n"/>
+      <c r="B89" s="11" t="inlineStr">
+        <is>
+          <t>E2E-004</t>
+        </is>
+      </c>
+      <c r="C89" s="11" t="inlineStr">
+        <is>
+          <t>npm run test:e2e</t>
+        </is>
+      </c>
+      <c r="D89" s="11">
+        <f>PROPER(G89)</f>
+        <v/>
+      </c>
+      <c r="E89" s="11">
+        <f>PROPER(H89)</f>
+        <v/>
+      </c>
+      <c r="F89" s="12" t="inlineStr">
+        <is>
+          <t>e2e/player-journeys.spec.ts
+• Database running and seeded (npm run seed:competition)
+• npm run test:e2e starts the backend and frontend if they are not running</t>
+        </is>
+      </c>
+      <c r="G89" s="11" t="inlineStr">
+        <is>
           <t>see my competitions</t>
         </is>
       </c>
-      <c r="H85" s="11" t="inlineStr">
+      <c r="H89" s="11" t="inlineStr">
         <is>
           <t>test data is seeded</t>
         </is>
       </c>
-      <c r="I85" s="12" t="inlineStr">
+      <c r="I89" s="12" t="inlineStr">
         <is>
           <t>• Log in as chloe.cooper005@players.example / WaverleyDev#2026
 • Open Competitions: Weekend Senior is listed as an active entry
@@ -3370,50 +3508,50 @@
 • Open Past seasons: Night Tennis and Glen Waverley A are listed</t>
         </is>
       </c>
-      <c r="J85" s="11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="13" t="n"/>
-      <c r="B87" s="11" t="inlineStr">
+      <c r="J89" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="13" t="n"/>
+      <c r="B91" s="11" t="inlineStr">
         <is>
           <t>E2E-005</t>
         </is>
       </c>
-      <c r="C87" s="11" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D87" s="11">
-        <f>PROPER(G87)</f>
-        <v/>
-      </c>
-      <c r="E87" s="11">
-        <f>PROPER(H87)</f>
-        <v/>
-      </c>
-      <c r="F87" s="12" t="inlineStr">
-        <is>
-          <t>• Database running and seeded (npm run seed:competition)
-• npm run dev:backend and npm run dev:frontend
-• Open http://localhost:5173</t>
-        </is>
-      </c>
-      <c r="G87" s="11" t="inlineStr">
+      <c r="C91" s="11" t="inlineStr">
+        <is>
+          <t>npm run test:e2e</t>
+        </is>
+      </c>
+      <c r="D91" s="11">
+        <f>PROPER(G91)</f>
+        <v/>
+      </c>
+      <c r="E91" s="11">
+        <f>PROPER(H91)</f>
+        <v/>
+      </c>
+      <c r="F91" s="12" t="inlineStr">
+        <is>
+          <t>e2e/player-journeys.spec.ts
+• Database running and seeded (npm run seed:competition)
+• npm run test:e2e starts the backend and frontend if they are not running</t>
+        </is>
+      </c>
+      <c r="G91" s="11" t="inlineStr">
         <is>
           <t>see my fixtures and results</t>
         </is>
       </c>
-      <c r="H87" s="11" t="inlineStr">
+      <c r="H91" s="11" t="inlineStr">
         <is>
           <t>test data is seeded</t>
         </is>
       </c>
-      <c r="I87" s="12" t="inlineStr">
+      <c r="I91" s="12" t="inlineStr">
         <is>
           <t>• Log in as chloe.cooper005@players.example / WaverleyDev#2026
 • Open Matches: upcoming fixtures are listed
@@ -3421,50 +3559,50 @@
 • Open History, then View scorecard, and check the set scores</t>
         </is>
       </c>
-      <c r="J87" s="11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="13" t="n"/>
-      <c r="B89" s="11" t="inlineStr">
+      <c r="J91" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="13" t="n"/>
+      <c r="B93" s="11" t="inlineStr">
         <is>
           <t>E2E-006</t>
         </is>
       </c>
-      <c r="C89" s="11" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D89" s="11">
-        <f>PROPER(G89)</f>
-        <v/>
-      </c>
-      <c r="E89" s="11">
-        <f>PROPER(H89)</f>
-        <v/>
-      </c>
-      <c r="F89" s="12" t="inlineStr">
-        <is>
-          <t>• Database running and seeded (npm run seed:competition)
-• npm run dev:backend and npm run dev:frontend
-• Open http://localhost:5173</t>
-        </is>
-      </c>
-      <c r="G89" s="11" t="inlineStr">
+      <c r="C93" s="11" t="inlineStr">
+        <is>
+          <t>npm run test:e2e</t>
+        </is>
+      </c>
+      <c r="D93" s="11">
+        <f>PROPER(G93)</f>
+        <v/>
+      </c>
+      <c r="E93" s="11">
+        <f>PROPER(H93)</f>
+        <v/>
+      </c>
+      <c r="F93" s="12" t="inlineStr">
+        <is>
+          <t>e2e/player-journeys.spec.ts
+• Database running and seeded (npm run seed:competition)
+• npm run test:e2e starts the backend and frontend if they are not running</t>
+        </is>
+      </c>
+      <c r="G93" s="11" t="inlineStr">
         <is>
           <t>see my clubs and team members</t>
         </is>
       </c>
-      <c r="H89" s="11" t="inlineStr">
+      <c r="H93" s="11" t="inlineStr">
         <is>
           <t>test data is seeded</t>
         </is>
       </c>
-      <c r="I89" s="12" t="inlineStr">
+      <c r="I93" s="12" t="inlineStr">
         <is>
           <t>• Log in as chloe.cooper005@players.example / WaverleyDev#2026
 • Open My Clubs: 2 associations, 4 clubs, 3 teams
@@ -3472,156 +3610,156 @@
 • Check the roster marks you with a You tag</t>
         </is>
       </c>
-      <c r="J89" s="11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="13" t="n"/>
-      <c r="B91" s="11" t="inlineStr">
+      <c r="J93" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="13" t="n"/>
+      <c r="B95" s="11" t="inlineStr">
         <is>
           <t>E2E-007</t>
         </is>
       </c>
-      <c r="C91" s="11" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D91" s="11">
-        <f>PROPER(G91)</f>
-        <v/>
-      </c>
-      <c r="E91" s="11">
-        <f>PROPER(H91)</f>
-        <v/>
-      </c>
-      <c r="F91" s="12" t="inlineStr">
-        <is>
-          <t>• Database running and seeded (npm run seed:competition)
-• npm run dev:backend and npm run dev:frontend
-• Open http://localhost:5173</t>
-        </is>
-      </c>
-      <c r="G91" s="11" t="inlineStr">
+      <c r="C95" s="11" t="inlineStr">
+        <is>
+          <t>npm run test:e2e</t>
+        </is>
+      </c>
+      <c r="D95" s="11">
+        <f>PROPER(G95)</f>
+        <v/>
+      </c>
+      <c r="E95" s="11">
+        <f>PROPER(H95)</f>
+        <v/>
+      </c>
+      <c r="F95" s="12" t="inlineStr">
+        <is>
+          <t>e2e/player-journeys.spec.ts
+• Database running and seeded (npm run seed:competition)
+• npm run test:e2e starts the backend and frontend if they are not running</t>
+        </is>
+      </c>
+      <c r="G95" s="11" t="inlineStr">
         <is>
           <t>check standings and rankings</t>
         </is>
       </c>
-      <c r="H91" s="11" t="inlineStr">
+      <c r="H95" s="11" t="inlineStr">
         <is>
           <t>test data is seeded</t>
         </is>
       </c>
-      <c r="I91" s="12" t="inlineStr">
+      <c r="I95" s="12" t="inlineStr">
         <is>
           <t>• Log in as chloe.cooper005@players.example / WaverleyDev#2026
 • Open Standings &amp; Rankings: your team and your position are highlighted
 • Switch to the UTR rankings tab and check the Better than N% column</t>
         </is>
       </c>
-      <c r="J91" s="11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="13" t="n"/>
-      <c r="B93" s="11" t="inlineStr">
+      <c r="J95" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="13" t="n"/>
+      <c r="B97" s="11" t="inlineStr">
         <is>
           <t>E2E-008</t>
         </is>
       </c>
-      <c r="C93" s="11" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D93" s="11">
-        <f>PROPER(G93)</f>
-        <v/>
-      </c>
-      <c r="E93" s="11">
-        <f>PROPER(H93)</f>
-        <v/>
-      </c>
-      <c r="F93" s="12" t="inlineStr">
-        <is>
-          <t>• Database running and seeded (npm run seed:competition)
-• npm run dev:backend and npm run dev:frontend
-• Open http://localhost:5173</t>
-        </is>
-      </c>
-      <c r="G93" s="11" t="inlineStr">
+      <c r="C97" s="11" t="inlineStr">
+        <is>
+          <t>npm run test:e2e</t>
+        </is>
+      </c>
+      <c r="D97" s="11">
+        <f>PROPER(G97)</f>
+        <v/>
+      </c>
+      <c r="E97" s="11">
+        <f>PROPER(H97)</f>
+        <v/>
+      </c>
+      <c r="F97" s="12" t="inlineStr">
+        <is>
+          <t>e2e/player-journeys.spec.ts
+• Database running and seeded (npm run seed:competition)
+• npm run test:e2e starts the backend and frontend if they are not running</t>
+        </is>
+      </c>
+      <c r="G97" s="11" t="inlineStr">
         <is>
           <t>find who to contact</t>
         </is>
       </c>
-      <c r="H93" s="11" t="inlineStr">
+      <c r="H97" s="11" t="inlineStr">
         <is>
           <t>test data is seeded</t>
         </is>
       </c>
-      <c r="I93" s="12" t="inlineStr">
+      <c r="I97" s="12" t="inlineStr">
         <is>
           <t>• Log in as chloe.cooper005@players.example / WaverleyDev#2026
 • Open Help &amp; Support
 • Check the team manager, club administrator and records secretary are named</t>
         </is>
       </c>
-      <c r="J93" s="11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="13" t="n"/>
-      <c r="B95" s="11" t="inlineStr">
+      <c r="J97" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="13" t="n"/>
+      <c r="B99" s="11" t="inlineStr">
         <is>
           <t>E2E-009</t>
         </is>
       </c>
-      <c r="C95" s="11" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="D95" s="11">
-        <f>PROPER(G95)</f>
-        <v/>
-      </c>
-      <c r="E95" s="11">
-        <f>PROPER(H95)</f>
-        <v/>
-      </c>
-      <c r="F95" s="12" t="inlineStr">
-        <is>
-          <t>• Database running and seeded (npm run seed:competition)
-• npm run dev:backend and npm run dev:frontend
-• Open http://localhost:5173</t>
-        </is>
-      </c>
-      <c r="G95" s="11" t="inlineStr">
+      <c r="C99" s="11" t="inlineStr">
+        <is>
+          <t>npm run test:e2e</t>
+        </is>
+      </c>
+      <c r="D99" s="11">
+        <f>PROPER(G99)</f>
+        <v/>
+      </c>
+      <c r="E99" s="11">
+        <f>PROPER(H99)</f>
+        <v/>
+      </c>
+      <c r="F99" s="12" t="inlineStr">
+        <is>
+          <t>e2e/player-journeys.spec.ts
+• Database running and seeded (npm run seed:competition)
+• npm run test:e2e starts the backend and frontend if they are not running</t>
+        </is>
+      </c>
+      <c r="G99" s="11" t="inlineStr">
         <is>
           <t>preview the site without logging in</t>
         </is>
       </c>
-      <c r="H95" s="11" t="inlineStr">
+      <c r="H99" s="11" t="inlineStr">
         <is>
           <t>test data is seeded</t>
         </is>
       </c>
-      <c r="I95" s="12" t="inlineStr">
+      <c r="I99" s="12" t="inlineStr">
         <is>
           <t>• Without logging in, open http://localhost:5173/dashboard
 • Check the sample player Chloe Cooper is shown on every page</t>
         </is>
       </c>
-      <c r="J95" s="11" t="inlineStr">
+      <c r="J99" s="11" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>